<commit_message>
Deploying to gh-pages from  @ fae75b130d41458b96ae9a19563106809d4adcf3 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/AidType.xlsx
+++ b/api/clv1/codelist/AidType.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="89">
   <si>
     <t>code</t>
   </si>
@@ -103,6 +103,33 @@
     <t>In addition to their core-funded operations, international organisations, NGOs, PPPs and networks, both in provider and in third countries, set up programmes and funds with a specific sectoral, thematic or geographical focus. Donors’ bilateral contributions to such programmes and funds are recorded here.</t>
   </si>
   <si>
+    <t>B031</t>
+  </si>
+  <si>
+    <t>Contributions to multi-donor/multi-entity funding mechanisms</t>
+  </si>
+  <si>
+    <t>Funding mechanisms that pool contributions from several donors and that are implemented by several multilateral entities e.g. UN inter-agency pooled funds, including CERF and country-based pooled funds; Financial Intermediary Funds (GEF, CIFs) for which the World Bank is the Trustee.</t>
+  </si>
+  <si>
+    <t>B032</t>
+  </si>
+  <si>
+    <t>Contributions to multi-donor/single-entity funding mechanisms</t>
+  </si>
+  <si>
+    <t>Contributions to multi-donor funding mechanisms managed by a single multilateral organisation e.g. UN single-agency thematic funds; World Bank or other MDB trust funds. Classify the contribution as B032 even if in the initial stages only one donor contributes to the fund.</t>
+  </si>
+  <si>
+    <t>B033</t>
+  </si>
+  <si>
+    <t>Contributions to single-donor funding mechanisms and contributions earmarked for a specific funding window or geographical location</t>
+  </si>
+  <si>
+    <t>Contributions to funding mechanisms where the donor has a significant influence on the allocation of funds. This includes contributions to single-donor trust funds and earmarked contributions to specific countries/geographical locations or funding windows within multi-donor trust funds. When the donor designs the activity but channels it through an international organisation, the activity should be classified as C01.</t>
+  </si>
+  <si>
     <t>B04</t>
   </si>
   <si>
@@ -118,7 +145,7 @@
     <t>Project-type interventions</t>
   </si>
   <si>
-    <t>A project is a set of inputs, activities and outputs, agreed with the partner country*, to reach specific objectives/outcomes within a defined time frame, with a defined budget and a  defined geographical area. Projects can vary significantly in terms of objectives, complexity, amounts involved and duration. There are smaller projects that might involve modest financial resources and last only a few months, whereas large projects might involve more significant amounts, entail successive phases and last for many years. A large project with a number of different components is sometimes referred to as a programme, but should nevertheless be recorded here. Feasibility studies, appraisals and evaluations are included (whether designed as part of projects/programmes or dedicated funding arrangements). Academic studies, research and development, trainings, scholarships, and other technical assistance activities not directly linked to development projects/programmes should instead be recorded under D02. Aid channelled through NGOs or multilaterals is also recorded here. This includes payments for NGOs and multilaterals to implement donors’ projects and programmes, and funding of specified NGOs projects. By contrast, core funding of NGOs and multilaterals as well as contributions to specific-purpose funds are recorded under B.* In the cases of equity investments, humanitarian aid or aid channelled through NGOs, projects are recorded here even if there was no direct agreement between the donor and the partner country.</t>
+    <t>A project is a set of inputs, activities and outputs, agreed with the partner country*, to reach specific objectives/outcomes within a defined time frame, with a defined budget and a  defined geographical area. Projects can vary significantly in terms of objectives, complexity, amounts involved and duration. There are smaller projects that might involve modest financial resources and last only a few months, whereas large projects might involve more significant amounts, entail successive phases and last for many years. A large project with a number of different components is sometimes referred to as a programme, but should nevertheless be recorded here. Feasibility studies, appraisals and evaluations are included (whether designed as part of projects/programmes or dedicated funding arrangements). Academic studies, research and development, trainings, scholarships, and other technical assistance activities not directly linked to development projects/programmes should instead be recorded under D02. Aid channelled through NGOs or multilaterals is also recorded here. This includes payments for NGOs and multilaterals to implement donors’ projects and programmes, and funding of specified NGOs projects. By contrast, core funding of NGOs and multilaterals as well as contributions to specific-purpose funds are recorded under B.* In the cases of equity investments, humanitarian aid or aid channelled through NGOs, projects are recorded here even if there was no direct agreement between the donor and the partner country. Contributions to single-donor trust funds and contributions to trust funds earmarked for a specific funding window and/or country are recorded under B033.</t>
   </si>
   <si>
     <t>C</t>
@@ -585,7 +612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -740,13 +767,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -763,90 +784,81 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" t="s">
-        <v>41</v>
-      </c>
-      <c r="G9" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>42</v>
+      </c>
+      <c r="G11" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
@@ -857,42 +869,48 @@
       <c r="F12" t="s">
         <v>50</v>
       </c>
+      <c r="G12" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" t="s">
         <v>54</v>
       </c>
-      <c r="B13" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" t="s">
-        <v>56</v>
-      </c>
       <c r="D13" t="s">
         <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="F13" t="s">
-        <v>55</v>
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
         <v>58</v>
-      </c>
-      <c r="B14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" t="s">
-        <v>61</v>
       </c>
       <c r="F14" t="s">
         <v>59</v>
@@ -900,94 +918,85 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" t="s">
         <v>62</v>
       </c>
-      <c r="B15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" t="s">
-        <v>64</v>
-      </c>
       <c r="D15" t="s">
         <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
-      </c>
-      <c r="G15" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
-      </c>
-      <c r="G16" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F17" t="s">
-        <v>66</v>
-      </c>
-      <c r="G17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
         <v>74</v>
       </c>
-      <c r="B18" t="s">
+      <c r="F18" t="s">
         <v>75</v>
       </c>
-      <c r="C18" t="s">
+      <c r="G18" t="s">
         <v>76</v>
-      </c>
-      <c r="D18" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" t="s">
-        <v>65</v>
-      </c>
-      <c r="F18" t="s">
-        <v>66</v>
-      </c>
-      <c r="G18" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1004,13 +1013,82 @@
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F19" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s">
+        <v>74</v>
+      </c>
+      <c r="F20" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" t="s">
+        <v>75</v>
+      </c>
+      <c r="G21" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>